<commit_message>
FH(UpdateData): Update data and fix issues
</commit_message>
<xml_diff>
--- a/ressources/budget.xlsx
+++ b/ressources/budget.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="actuel" sheetId="1" state="visible" r:id="rId3"/>
@@ -653,7 +653,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I107"/>
-  <sheetFormatPr defaultColWidth="15.12890625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.12890625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="19.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="6.63"/>
@@ -1755,7 +1755,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:I53"/>
-  <sheetFormatPr defaultColWidth="15.12890625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.12890625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="18.36"/>
+  </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
@@ -1793,7 +1796,7 @@
       </c>
       <c r="C2" s="9" t="n">
         <f aca="false">SUM(C6:C51)</f>
-        <v>2762.5</v>
+        <v>3190.5</v>
       </c>
       <c r="D2" s="10" t="n">
         <f aca="false">D5</f>
@@ -1801,7 +1804,7 @@
       </c>
       <c r="E2" s="11" t="n">
         <f aca="false">SUM(E6:E102)</f>
-        <v>33150</v>
+        <v>38286</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1818,7 +1821,7 @@
       </c>
       <c r="C4" s="17" t="n">
         <f aca="false">B2-C2</f>
-        <v>437.5</v>
+        <v>9.5</v>
       </c>
       <c r="D4" s="14"/>
       <c r="E4" s="18"/>
@@ -1865,12 +1868,12 @@
         <v>9</v>
       </c>
       <c r="C7" s="24" t="n">
-        <v>600</v>
+        <v>800</v>
       </c>
       <c r="D7" s="21"/>
       <c r="E7" s="22" t="n">
         <f aca="false">C7*12</f>
-        <v>7200</v>
+        <v>9600</v>
       </c>
       <c r="F7" s="25" t="n">
         <v>442.841666666667</v>
@@ -1957,12 +1960,12 @@
         <v>13</v>
       </c>
       <c r="C11" s="24" t="n">
-        <v>0</v>
+        <v>118</v>
       </c>
       <c r="D11" s="21"/>
       <c r="E11" s="22" t="n">
         <f aca="false">C11*12</f>
-        <v>0</v>
+        <v>1416</v>
       </c>
       <c r="F11" s="25" t="n">
         <v>47.2775</v>
@@ -2187,12 +2190,12 @@
         <v>23</v>
       </c>
       <c r="C21" s="24" t="n">
-        <v>950</v>
+        <v>1060</v>
       </c>
       <c r="D21" s="21"/>
       <c r="E21" s="22" t="n">
         <f aca="false">C21*12</f>
-        <v>11400</v>
+        <v>12720</v>
       </c>
       <c r="F21" s="25" t="n">
         <v>772.323333333333</v>
@@ -2542,7 +2545,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:E16"/>
-  <sheetFormatPr defaultColWidth="15.12890625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="15.12890625" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="6.88"/>

</xml_diff>